<commit_message>
Scraper robusto (retry, emittenti indipendenti) e job schedulato con commit/push automatico
</commit_message>
<xml_diff>
--- a/data/rendimenti_etf.xlsx
+++ b/data/rendimenti_etf.xlsx
@@ -533,7 +533,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Aggiornato il 06/10/2026 09:16 da yield_etf.xlsx</t>
+          <t>Aggiornato il 07/10/2026 10:56 da yield_etf.csv</t>
         </is>
       </c>
     </row>
@@ -658,13 +658,13 @@
         <v/>
       </c>
       <c r="H5" s="8" t="n">
-        <v>0.0389</v>
+        <v>0.039</v>
       </c>
       <c r="I5" s="8" t="n">
-        <v>0.05019999999999999</v>
+        <v>0.0506</v>
       </c>
       <c r="J5" s="9" t="n">
-        <v>0</v>
+        <v>0.0004</v>
       </c>
       <c r="K5" s="9" t="n"/>
       <c r="L5" s="9" t="n"/>
@@ -724,10 +724,10 @@
         <v>0.03759999999999999</v>
       </c>
       <c r="I6" s="8" t="n">
-        <v>0.04650000000000001</v>
+        <v>0.0469</v>
       </c>
       <c r="J6" s="9" t="n">
-        <v>-0.0002</v>
+        <v>0.0004</v>
       </c>
       <c r="K6" s="9" t="n"/>
       <c r="L6" s="9" t="n"/>
@@ -747,7 +747,7 @@
         <v/>
       </c>
       <c r="Q6" s="12" t="n">
-        <v>28.21</v>
+        <v>28.34</v>
       </c>
     </row>
     <row r="7">
@@ -784,13 +784,13 @@
         <v/>
       </c>
       <c r="H7" s="8" t="n">
-        <v>0.0354</v>
+        <v>0.0355</v>
       </c>
       <c r="I7" s="8" t="n">
-        <v>0.0462</v>
+        <v>0.0466</v>
       </c>
       <c r="J7" s="9" t="n">
-        <v>0</v>
+        <v>0.0004</v>
       </c>
       <c r="K7" s="9" t="n"/>
       <c r="L7" s="9" t="n"/>
@@ -810,7 +810,7 @@
         <v/>
       </c>
       <c r="Q7" s="12" t="n">
-        <v>4.79</v>
+        <v>4.81</v>
       </c>
     </row>
     <row r="8">
@@ -850,10 +850,10 @@
         <v>0.0365</v>
       </c>
       <c r="I8" s="8" t="n">
-        <v>0.0461</v>
+        <v>0.04650000000000001</v>
       </c>
       <c r="J8" s="9" t="n">
-        <v>0.0206</v>
+        <v>0.0004</v>
       </c>
       <c r="K8" s="9" t="n"/>
       <c r="L8" s="9" t="n"/>
@@ -873,7 +873,7 @@
         <v/>
       </c>
       <c r="Q8" s="12" t="n">
-        <v>29.04</v>
+        <v>29.15</v>
       </c>
     </row>
     <row r="9">
@@ -913,10 +913,10 @@
         <v>0.0349</v>
       </c>
       <c r="I9" s="8" t="n">
-        <v>0.0459</v>
+        <v>0.0464</v>
       </c>
       <c r="J9" s="9" t="n">
-        <v>0</v>
+        <v>0.0005</v>
       </c>
       <c r="K9" s="9" t="n"/>
       <c r="L9" s="9" t="n"/>
@@ -936,7 +936,7 @@
         <v/>
       </c>
       <c r="Q9" s="12" t="n">
-        <v>4.79</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="10">
@@ -976,10 +976,10 @@
         <v>0.0363</v>
       </c>
       <c r="I10" s="8" t="n">
-        <v>0.0458</v>
+        <v>0.0463</v>
       </c>
       <c r="J10" s="9" t="n">
-        <v>0</v>
+        <v>0.0005</v>
       </c>
       <c r="K10" s="9" t="n"/>
       <c r="L10" s="9" t="n"/>
@@ -999,7 +999,7 @@
         <v/>
       </c>
       <c r="Q10" s="12" t="n">
-        <v>4.71</v>
+        <v>4.72</v>
       </c>
     </row>
     <row r="11">
@@ -1039,10 +1039,10 @@
         <v>0.0347</v>
       </c>
       <c r="I11" s="8" t="n">
-        <v>0.0455</v>
+        <v>0.0459</v>
       </c>
       <c r="J11" s="9" t="n">
-        <v>0</v>
+        <v>0.0004</v>
       </c>
       <c r="K11" s="9" t="n"/>
       <c r="L11" s="9" t="n"/>
@@ -1062,7 +1062,7 @@
         <v/>
       </c>
       <c r="Q11" s="12" t="n">
-        <v>33.42</v>
+        <v>33.53</v>
       </c>
     </row>
     <row r="12">
@@ -1099,13 +1099,13 @@
         <v/>
       </c>
       <c r="H12" s="8" t="n">
-        <v>0.0347</v>
+        <v>0.0346</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>0.045</v>
+        <v>0.0454</v>
       </c>
       <c r="J12" s="9" t="n">
-        <v>0</v>
+        <v>0.0004</v>
       </c>
       <c r="K12" s="9" t="n"/>
       <c r="L12" s="9" t="n"/>
@@ -1125,7 +1125,7 @@
         <v/>
       </c>
       <c r="Q12" s="12" t="n">
-        <v>4.72</v>
+        <v>4.75</v>
       </c>
     </row>
     <row r="13">
@@ -1165,10 +1165,10 @@
         <v>0.034</v>
       </c>
       <c r="I13" s="8" t="n">
-        <v>0.0447</v>
+        <v>0.0451</v>
       </c>
       <c r="J13" s="9" t="n">
-        <v>0.0196</v>
+        <v>0.0004</v>
       </c>
       <c r="K13" s="9" t="n"/>
       <c r="L13" s="9" t="n"/>
@@ -1188,7 +1188,7 @@
         <v/>
       </c>
       <c r="Q13" s="12" t="n">
-        <v>9.279999999999999</v>
+        <v>9.31</v>
       </c>
     </row>
     <row r="14">
@@ -1228,10 +1228,10 @@
         <v>0.034</v>
       </c>
       <c r="I14" s="8" t="n">
-        <v>0.0447</v>
+        <v>0.0451</v>
       </c>
       <c r="J14" s="9" t="n">
-        <v>0.0196</v>
+        <v>0.0004</v>
       </c>
       <c r="K14" s="9" t="n"/>
       <c r="L14" s="9" t="n"/>
@@ -1251,7 +1251,7 @@
         <v/>
       </c>
       <c r="Q14" s="12" t="n">
-        <v>27.81</v>
+        <v>27.9</v>
       </c>
     </row>
     <row r="15">
@@ -1288,13 +1288,13 @@
         <v/>
       </c>
       <c r="H15" s="8" t="n">
-        <v>0.0332</v>
+        <v>0.0331</v>
       </c>
       <c r="I15" s="8" t="n">
-        <v>0.0443</v>
+        <v>0.0447</v>
       </c>
       <c r="J15" s="9" t="n">
-        <v>0</v>
+        <v>0.0004</v>
       </c>
       <c r="K15" s="9" t="n"/>
       <c r="L15" s="9" t="n"/>
@@ -1314,7 +1314,7 @@
         <v/>
       </c>
       <c r="Q15" s="12" t="n">
-        <v>4.76</v>
+        <v>4.77</v>
       </c>
     </row>
     <row r="16">
@@ -1354,10 +1354,10 @@
         <v>0.0282</v>
       </c>
       <c r="I16" s="8" t="n">
-        <v>0.0438</v>
+        <v>0.0441</v>
       </c>
       <c r="J16" s="9" t="n">
-        <v>0.0001</v>
+        <v>0.0003</v>
       </c>
       <c r="K16" s="9" t="n"/>
       <c r="L16" s="9" t="n"/>
@@ -1377,7 +1377,7 @@
         <v/>
       </c>
       <c r="Q16" s="12" t="n">
-        <v>34.2</v>
+        <v>34.29</v>
       </c>
     </row>
     <row r="17">
@@ -1414,13 +1414,13 @@
         <v/>
       </c>
       <c r="H17" s="8" t="n">
-        <v>0.0336</v>
+        <v>0.0335</v>
       </c>
       <c r="I17" s="8" t="n">
-        <v>0.0445</v>
+        <v>0.04480000000000001</v>
       </c>
       <c r="J17" s="9" t="n">
-        <v>0</v>
+        <v>0.0003</v>
       </c>
       <c r="K17" s="9" t="n"/>
       <c r="L17" s="9" t="n"/>
@@ -1440,7 +1440,7 @@
         <v/>
       </c>
       <c r="Q17" s="12" t="n">
-        <v>5.09</v>
+        <v>5.1</v>
       </c>
     </row>
     <row r="18">
@@ -1477,13 +1477,13 @@
         <v/>
       </c>
       <c r="H18" s="8" t="n">
-        <v>0.0299</v>
+        <v>0.03</v>
       </c>
       <c r="I18" s="8" t="n">
-        <v>0.043</v>
+        <v>0.0435</v>
       </c>
       <c r="J18" s="9" t="n">
-        <v>0</v>
+        <v>0.0005</v>
       </c>
       <c r="K18" s="9" t="n"/>
       <c r="L18" s="9" t="n"/>
@@ -1503,7 +1503,7 @@
         <v/>
       </c>
       <c r="Q18" s="12" t="n">
-        <v>4.81</v>
+        <v>4.82</v>
       </c>
     </row>
     <row r="19">
@@ -1543,10 +1543,10 @@
         <v>0.0169</v>
       </c>
       <c r="I19" s="8" t="n">
-        <v>0.0362</v>
+        <v>0.0365</v>
       </c>
       <c r="J19" s="9" t="n">
-        <v>-0.0004</v>
+        <v>0.0003</v>
       </c>
       <c r="K19" s="9" t="n"/>
       <c r="L19" s="9" t="n"/>
@@ -1566,7 +1566,7 @@
         <v/>
       </c>
       <c r="Q19" s="12" t="n">
-        <v>9.8202</v>
+        <v>9.844900000000001</v>
       </c>
     </row>
     <row r="20">
@@ -1603,13 +1603,13 @@
         <v/>
       </c>
       <c r="H20" s="8" t="n">
-        <v>0.0284</v>
+        <v>0.0285</v>
       </c>
       <c r="I20" s="8" t="n">
-        <v>0.0424</v>
+        <v>0.0428</v>
       </c>
       <c r="J20" s="9" t="n">
-        <v>0</v>
+        <v>0.0004</v>
       </c>
       <c r="K20" s="9" t="n"/>
       <c r="L20" s="9" t="n"/>
@@ -1669,10 +1669,10 @@
         <v>0.0269</v>
       </c>
       <c r="I21" s="8" t="n">
-        <v>0.0424</v>
+        <v>0.04269999999999999</v>
       </c>
       <c r="J21" s="9" t="n">
-        <v>0</v>
+        <v>0.0003</v>
       </c>
       <c r="K21" s="9" t="n"/>
       <c r="L21" s="9" t="n"/>
@@ -1692,7 +1692,7 @@
         <v/>
       </c>
       <c r="Q21" s="12" t="n">
-        <v>10.4073</v>
+        <v>10.3893</v>
       </c>
     </row>
     <row r="22">
@@ -1732,10 +1732,10 @@
         <v>0.0269</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>0.0424</v>
+        <v>0.04269999999999999</v>
       </c>
       <c r="J22" s="9" t="n">
-        <v>0</v>
+        <v>0.0003</v>
       </c>
       <c r="K22" s="9" t="n"/>
       <c r="L22" s="9" t="n"/>
@@ -1755,23 +1755,23 @@
         <v/>
       </c>
       <c r="Q22" s="12" t="n">
-        <v>10.0222</v>
+        <v>10.0049</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Invesco</t>
+          <t>DWS</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Invesco BulletShares 2030 EUR Corporate Bond UCITS ETF Acc</t>
+          <t>Xtrackers II Target Maturity Sept 2031 EUR Corporate Bond UCITS ETF 1C</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>IE000I25S1V5</t>
+          <t>LU2673523135</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
@@ -1785,7 +1785,7 @@
         </is>
       </c>
       <c r="F23" s="6" t="n">
-        <v>47848</v>
+        <v>48121</v>
       </c>
       <c r="G23" s="7">
         <f>IF(F23="","",MAX(0,YEARFRAC(TODAY(),F23)))</f>
@@ -1795,15 +1795,15 @@
         <v>0.0287</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>0.0421</v>
+        <v>0.0424</v>
       </c>
       <c r="J23" s="9" t="n">
-        <v>0</v>
+        <v>0.0004</v>
       </c>
       <c r="K23" s="9" t="n"/>
       <c r="L23" s="9" t="n"/>
       <c r="M23" s="8" t="n">
-        <v>0.001</v>
+        <v>0.0012</v>
       </c>
       <c r="N23" s="10">
         <f>IF(D23="Govt",$B$1,$B$2)</f>
@@ -1818,23 +1818,23 @@
         <v/>
       </c>
       <c r="Q23" s="12" t="n">
-        <v>5.34</v>
+        <v>9.789999999999999</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Invesco</t>
+          <t>DWS</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Invesco BulletShares 2030 EUR Corporate Bond UCITS ETF Dist</t>
+          <t>Xtrackers II Target Maturity Sept 2031 EUR Corporate Bond UCITS ETF 1D</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>IE000W6YTDH7</t>
+          <t>LU2673523481</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
@@ -1848,7 +1848,7 @@
         </is>
       </c>
       <c r="F24" s="6" t="n">
-        <v>47848</v>
+        <v>48121</v>
       </c>
       <c r="G24" s="7">
         <f>IF(F24="","",MAX(0,YEARFRAC(TODAY(),F24)))</f>
@@ -1858,15 +1858,15 @@
         <v>0.0287</v>
       </c>
       <c r="I24" s="8" t="n">
-        <v>0.0421</v>
+        <v>0.0424</v>
       </c>
       <c r="J24" s="9" t="n">
-        <v>0</v>
+        <v>0.0004</v>
       </c>
       <c r="K24" s="9" t="n"/>
       <c r="L24" s="9" t="n"/>
       <c r="M24" s="8" t="n">
-        <v>0.001</v>
+        <v>0.0012</v>
       </c>
       <c r="N24" s="10">
         <f>IF(D24="Govt",$B$1,$B$2)</f>
@@ -1881,23 +1881,23 @@
         <v/>
       </c>
       <c r="Q24" s="12" t="n">
-        <v>4.9741</v>
+        <v>29.28</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>DWS</t>
+          <t>Invesco</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Xtrackers II Target Maturity Sept 2031 EUR Corporate Bond UCITS ETF 1C</t>
+          <t>Invesco BulletShares 2030 EUR Corporate Bond UCITS ETF Acc</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>LU2673523135</t>
+          <t>IE000I25S1V5</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
@@ -1911,7 +1911,7 @@
         </is>
       </c>
       <c r="F25" s="6" t="n">
-        <v>48121</v>
+        <v>47848</v>
       </c>
       <c r="G25" s="7">
         <f>IF(F25="","",MAX(0,YEARFRAC(TODAY(),F25)))</f>
@@ -1921,15 +1921,15 @@
         <v>0.0287</v>
       </c>
       <c r="I25" s="8" t="n">
-        <v>0.042</v>
+        <v>0.0421</v>
       </c>
       <c r="J25" s="9" t="n">
-        <v>0.017</v>
+        <v>0</v>
       </c>
       <c r="K25" s="9" t="n"/>
       <c r="L25" s="9" t="n"/>
       <c r="M25" s="8" t="n">
-        <v>0.0012</v>
+        <v>0.001</v>
       </c>
       <c r="N25" s="10">
         <f>IF(D25="Govt",$B$1,$B$2)</f>
@@ -1944,23 +1944,23 @@
         <v/>
       </c>
       <c r="Q25" s="12" t="n">
-        <v>9.77</v>
+        <v>5.3502</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>DWS</t>
+          <t>Invesco</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Xtrackers II Target Maturity Sept 2031 EUR Corporate Bond UCITS ETF 1D</t>
+          <t>Invesco BulletShares 2030 EUR Corporate Bond UCITS ETF Dist</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>LU2673523481</t>
+          <t>IE000W6YTDH7</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
@@ -1974,7 +1974,7 @@
         </is>
       </c>
       <c r="F26" s="6" t="n">
-        <v>48121</v>
+        <v>47848</v>
       </c>
       <c r="G26" s="7">
         <f>IF(F26="","",MAX(0,YEARFRAC(TODAY(),F26)))</f>
@@ -1984,15 +1984,15 @@
         <v>0.0287</v>
       </c>
       <c r="I26" s="8" t="n">
-        <v>0.042</v>
+        <v>0.0421</v>
       </c>
       <c r="J26" s="9" t="n">
-        <v>0.017</v>
+        <v>0</v>
       </c>
       <c r="K26" s="9" t="n"/>
       <c r="L26" s="9" t="n"/>
       <c r="M26" s="8" t="n">
-        <v>0.0012</v>
+        <v>0.001</v>
       </c>
       <c r="N26" s="10">
         <f>IF(D26="Govt",$B$1,$B$2)</f>
@@ -2007,7 +2007,7 @@
         <v/>
       </c>
       <c r="Q26" s="12" t="n">
-        <v>29.25</v>
+        <v>4.9836</v>
       </c>
     </row>
     <row r="27">
@@ -2044,13 +2044,13 @@
         <v/>
       </c>
       <c r="H27" s="8" t="n">
-        <v>0.0208</v>
+        <v>0.0207</v>
       </c>
       <c r="I27" s="8" t="n">
-        <v>0.0353</v>
+        <v>0.0356</v>
       </c>
       <c r="J27" s="9" t="n">
-        <v>-0.0004</v>
+        <v>0.0003</v>
       </c>
       <c r="K27" s="9" t="n"/>
       <c r="L27" s="9" t="n"/>
@@ -2070,23 +2070,23 @@
         <v/>
       </c>
       <c r="Q27" s="12" t="n">
-        <v>9.976800000000001</v>
+        <v>9.9948</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>iShares</t>
+          <t>DWS</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>iShares iBonds Dec 2028 Term € Italy Govt Bond UCITS ETF</t>
+          <t>Xtrackers II Target Maturity Sept 2029 Italy and Spain Government Bond UCITS ETF 1C</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>IE000Q2EQ5K8</t>
+          <t>LU0484969463</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
@@ -2096,24 +2096,24 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>Dist</t>
+          <t>Acc</t>
         </is>
       </c>
       <c r="F28" s="6" t="n">
-        <v>47118</v>
+        <v>47391</v>
       </c>
       <c r="G28" s="7">
         <f>IF(F28="","",MAX(0,YEARFRAC(TODAY(),F28)))</f>
         <v/>
       </c>
       <c r="H28" s="8" t="n">
-        <v>0.026</v>
+        <v>0.0297</v>
       </c>
       <c r="I28" s="8" t="n">
-        <v>0.0347</v>
+        <v>0.0351</v>
       </c>
       <c r="J28" s="9" t="n">
-        <v>0</v>
+        <v>0.0004</v>
       </c>
       <c r="K28" s="9" t="n"/>
       <c r="L28" s="9" t="n"/>
@@ -2133,50 +2133,50 @@
         <v/>
       </c>
       <c r="Q28" s="12" t="n">
-        <v>5.05</v>
+        <v>204.61</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>DWS</t>
+          <t>iShares</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Xtrackers II Target Maturity Sept 2029 Italy and Spain Government Bond UCITS ETF 1C</t>
+          <t>iShares iBonds Dec 2030 Term € Corp UCITS ETF</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>LU0484969463</t>
+          <t>IE000LX17BP9</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Govt</t>
+          <t>Corp</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>Acc</t>
+          <t>Dist</t>
         </is>
       </c>
       <c r="F29" s="6" t="n">
-        <v>47391</v>
+        <v>47848</v>
       </c>
       <c r="G29" s="7">
         <f>IF(F29="","",MAX(0,YEARFRAC(TODAY(),F29)))</f>
         <v/>
       </c>
       <c r="H29" s="8" t="n">
-        <v>0.0297</v>
+        <v>0.0279</v>
       </c>
       <c r="I29" s="8" t="n">
-        <v>0.0347</v>
+        <v>0.04099999999999999</v>
       </c>
       <c r="J29" s="9" t="n">
-        <v>0.0089</v>
+        <v>0.0003</v>
       </c>
       <c r="K29" s="9" t="n"/>
       <c r="L29" s="9" t="n"/>
@@ -2196,23 +2196,23 @@
         <v/>
       </c>
       <c r="Q29" s="12" t="n">
-        <v>204.21</v>
+        <v>4.99</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>iShares</t>
+          <t>DWS</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>iShares iBonds Dec 2030 Term € Corp UCITS ETF</t>
+          <t>Xtrackers II Target Maturity Sept 2030 EUR Corporate Bond UCITS ETF 1D</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>IE000LX17BP9</t>
+          <t>LU2809864296</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
@@ -2226,20 +2226,20 @@
         </is>
       </c>
       <c r="F30" s="6" t="n">
-        <v>47848</v>
+        <v>47756</v>
       </c>
       <c r="G30" s="7">
         <f>IF(F30="","",MAX(0,YEARFRAC(TODAY(),F30)))</f>
         <v/>
       </c>
       <c r="H30" s="8" t="n">
-        <v>0.0279</v>
+        <v>0.0271</v>
       </c>
       <c r="I30" s="8" t="n">
-        <v>0.0407</v>
+        <v>0.0409</v>
       </c>
       <c r="J30" s="9" t="n">
-        <v>0</v>
+        <v>0.0003</v>
       </c>
       <c r="K30" s="9" t="n"/>
       <c r="L30" s="9" t="n"/>
@@ -2259,28 +2259,28 @@
         <v/>
       </c>
       <c r="Q30" s="12" t="n">
-        <v>4.98</v>
+        <v>35.23</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>DWS</t>
+          <t>Amundi</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Xtrackers II Target Maturity Sept 2030 EUR Corporate Bond UCITS ETF 1D</t>
+          <t>Amundi Fixed Maturity 2028 Euro Government Bond Yield + UCITS ETF Dist</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>LU2809864296</t>
+          <t>LU2780871666</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Corp</t>
+          <t>Govt</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -2289,25 +2289,25 @@
         </is>
       </c>
       <c r="F31" s="6" t="n">
-        <v>47756</v>
+        <v>47118</v>
       </c>
       <c r="G31" s="7">
         <f>IF(F31="","",MAX(0,YEARFRAC(TODAY(),F31)))</f>
         <v/>
       </c>
       <c r="H31" s="8" t="n">
-        <v>0.0271</v>
+        <v>0.0229</v>
       </c>
       <c r="I31" s="8" t="n">
-        <v>0.0406</v>
+        <v>0.0341</v>
       </c>
       <c r="J31" s="9" t="n">
-        <v>0.0002</v>
+        <v>0.0004</v>
       </c>
       <c r="K31" s="9" t="n"/>
       <c r="L31" s="9" t="n"/>
       <c r="M31" s="8" t="n">
-        <v>0.0012</v>
+        <v>0.0009</v>
       </c>
       <c r="N31" s="10">
         <f>IF(D31="Govt",$B$1,$B$2)</f>
@@ -2322,55 +2322,55 @@
         <v/>
       </c>
       <c r="Q31" s="12" t="n">
-        <v>35.2</v>
+        <v>10.2881</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Invesco</t>
+          <t>iShares</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Invesco BulletShares 2029 EUR Corporate Bond UCITS ETF Acc</t>
+          <t>iShares iBonds Dec 2028 Term € Italy Govt Bond UCITS ETF</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>IE000P5IB8I8</t>
+          <t>IE000Q2EQ5K8</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Corp</t>
+          <t>Govt</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>Acc</t>
+          <t>Dist</t>
         </is>
       </c>
       <c r="F32" s="6" t="n">
-        <v>47483</v>
+        <v>47118</v>
       </c>
       <c r="G32" s="7">
         <f>IF(F32="","",MAX(0,YEARFRAC(TODAY(),F32)))</f>
         <v/>
       </c>
       <c r="H32" s="8" t="n">
-        <v>0.0242</v>
+        <v>0.026</v>
       </c>
       <c r="I32" s="8" t="n">
-        <v>0.0398</v>
+        <v>0.0342</v>
       </c>
       <c r="J32" s="9" t="n">
-        <v>0</v>
+        <v>-0.0005</v>
       </c>
       <c r="K32" s="9" t="n"/>
       <c r="L32" s="9" t="n"/>
       <c r="M32" s="8" t="n">
-        <v>0.001</v>
+        <v>0.0012</v>
       </c>
       <c r="N32" s="10">
         <f>IF(D32="Govt",$B$1,$B$2)</f>
@@ -2385,7 +2385,7 @@
         <v/>
       </c>
       <c r="Q32" s="12" t="n">
-        <v>5.4204</v>
+        <v>5.06</v>
       </c>
     </row>
     <row r="33">
@@ -2396,12 +2396,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Invesco BulletShares 2029 EUR Corporate Bond UCITS ETF Dist</t>
+          <t>Invesco BulletShares 2029 EUR Corporate Bond UCITS ETF Acc</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>IE000ZC4C5Q1</t>
+          <t>IE000P5IB8I8</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
@@ -2411,7 +2411,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>Dist</t>
+          <t>Acc</t>
         </is>
       </c>
       <c r="F33" s="6" t="n">
@@ -2448,28 +2448,28 @@
         <v/>
       </c>
       <c r="Q33" s="12" t="n">
-        <v>5.0508</v>
+        <v>5.4257</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Amundi</t>
+          <t>Invesco</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Amundi Fixed Maturity 2028 Euro Government Bond Yield + UCITS ETF Dist</t>
+          <t>Invesco BulletShares 2029 EUR Corporate Bond UCITS ETF Dist</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>LU2780871666</t>
+          <t>IE000ZC4C5Q1</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Govt</t>
+          <t>Corp</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -2478,25 +2478,25 @@
         </is>
       </c>
       <c r="F34" s="6" t="n">
-        <v>47118</v>
+        <v>47483</v>
       </c>
       <c r="G34" s="7">
         <f>IF(F34="","",MAX(0,YEARFRAC(TODAY(),F34)))</f>
         <v/>
       </c>
       <c r="H34" s="8" t="n">
-        <v>0.023</v>
+        <v>0.0242</v>
       </c>
       <c r="I34" s="8" t="n">
-        <v>0.0337</v>
+        <v>0.0398</v>
       </c>
       <c r="J34" s="9" t="n">
-        <v>-0.0004</v>
+        <v>0</v>
       </c>
       <c r="K34" s="9" t="n"/>
       <c r="L34" s="9" t="n"/>
       <c r="M34" s="8" t="n">
-        <v>0.0009</v>
+        <v>0.001</v>
       </c>
       <c r="N34" s="10">
         <f>IF(D34="Govt",$B$1,$B$2)</f>
@@ -2511,7 +2511,7 @@
         <v/>
       </c>
       <c r="Q34" s="12" t="n">
-        <v>10.2802</v>
+        <v>5.0558</v>
       </c>
     </row>
     <row r="35">
@@ -2554,7 +2554,7 @@
         <v>0.0334</v>
       </c>
       <c r="J35" s="9" t="n">
-        <v>-0.0004</v>
+        <v>0</v>
       </c>
       <c r="K35" s="9" t="n"/>
       <c r="L35" s="9" t="n"/>
@@ -2574,7 +2574,7 @@
         <v/>
       </c>
       <c r="Q35" s="12" t="n">
-        <v>10.2711</v>
+        <v>10.2777</v>
       </c>
     </row>
     <row r="36">
@@ -2617,7 +2617,7 @@
         <v>0.0334</v>
       </c>
       <c r="J36" s="9" t="n">
-        <v>-0.0004</v>
+        <v>0</v>
       </c>
       <c r="K36" s="9" t="n"/>
       <c r="L36" s="9" t="n"/>
@@ -2637,7 +2637,7 @@
         <v/>
       </c>
       <c r="Q36" s="12" t="n">
-        <v>10.0706</v>
+        <v>10.0771</v>
       </c>
     </row>
     <row r="37">
@@ -2677,10 +2677,10 @@
         <v>0.0251</v>
       </c>
       <c r="I37" s="8" t="n">
-        <v>0.0388</v>
+        <v>0.039</v>
       </c>
       <c r="J37" s="9" t="n">
-        <v>0</v>
+        <v>0.0002</v>
       </c>
       <c r="K37" s="9" t="n"/>
       <c r="L37" s="9" t="n"/>
@@ -2700,7 +2700,7 @@
         <v/>
       </c>
       <c r="Q37" s="12" t="n">
-        <v>5.03</v>
+        <v>5.04</v>
       </c>
     </row>
     <row r="38">
@@ -2740,10 +2740,10 @@
         <v>0.0245</v>
       </c>
       <c r="I38" s="8" t="n">
-        <v>0.0385</v>
+        <v>0.0387</v>
       </c>
       <c r="J38" s="9" t="n">
-        <v>0.0132</v>
+        <v>0.0002</v>
       </c>
       <c r="K38" s="9" t="n"/>
       <c r="L38" s="9" t="n"/>
@@ -2763,7 +2763,7 @@
         <v/>
       </c>
       <c r="Q38" s="12" t="n">
-        <v>25.77</v>
+        <v>25.78</v>
       </c>
     </row>
     <row r="39">
@@ -2803,10 +2803,10 @@
         <v>0.0245</v>
       </c>
       <c r="I39" s="8" t="n">
-        <v>0.0385</v>
+        <v>0.0387</v>
       </c>
       <c r="J39" s="9" t="n">
-        <v>0.0132</v>
+        <v>0.0002</v>
       </c>
       <c r="K39" s="9" t="n"/>
       <c r="L39" s="9" t="n"/>
@@ -2826,23 +2826,23 @@
         <v/>
       </c>
       <c r="Q39" s="12" t="n">
-        <v>9.16</v>
+        <v>9.17</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Invesco</t>
+          <t>BNP Paribas</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Invesco BulletShares 2028 EUR Corporate Bond UCITS ETF Acc</t>
+          <t>BNP PARIBAS EASY ESG ENHANCED EUR CORP BOND DECEMBER 2029 UCITS ETF C</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>IE00079EUF59</t>
+          <t>LU2823896811</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
@@ -2856,25 +2856,25 @@
         </is>
       </c>
       <c r="F40" s="6" t="n">
-        <v>47118</v>
+        <v>47483</v>
       </c>
       <c r="G40" s="7">
         <f>IF(F40="","",MAX(0,YEARFRAC(TODAY(),F40)))</f>
         <v/>
       </c>
       <c r="H40" s="8" t="n">
-        <v>0.0242</v>
+        <v>0.0235</v>
       </c>
       <c r="I40" s="8" t="n">
-        <v>0.0383</v>
+        <v>0.0385</v>
       </c>
       <c r="J40" s="9" t="n">
-        <v>0</v>
+        <v>0.0002</v>
       </c>
       <c r="K40" s="9" t="n"/>
       <c r="L40" s="9" t="n"/>
       <c r="M40" s="8" t="n">
-        <v>0.001</v>
+        <v>0.0012</v>
       </c>
       <c r="N40" s="10">
         <f>IF(D40="Govt",$B$1,$B$2)</f>
@@ -2889,23 +2889,23 @@
         <v/>
       </c>
       <c r="Q40" s="12" t="n">
-        <v>5.5679</v>
+        <v>10.6511</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Invesco</t>
+          <t>BNP Paribas</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Invesco BulletShares 2028 EUR Corporate Bond UCITS ETF Dist</t>
+          <t>BNP PARIBAS EASY ESG ENHANCED EUR CORP BOND DECEMBER 2029 UCITS ETF D</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>IE000LKGEZQ6</t>
+          <t>LU2823896738</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
@@ -2919,25 +2919,25 @@
         </is>
       </c>
       <c r="F41" s="6" t="n">
-        <v>47118</v>
+        <v>47483</v>
       </c>
       <c r="G41" s="7">
         <f>IF(F41="","",MAX(0,YEARFRAC(TODAY(),F41)))</f>
         <v/>
       </c>
       <c r="H41" s="8" t="n">
-        <v>0.0242</v>
+        <v>0.0235</v>
       </c>
       <c r="I41" s="8" t="n">
-        <v>0.0383</v>
+        <v>0.0385</v>
       </c>
       <c r="J41" s="9" t="n">
-        <v>0</v>
+        <v>0.0002</v>
       </c>
       <c r="K41" s="9" t="n"/>
       <c r="L41" s="9" t="n"/>
       <c r="M41" s="8" t="n">
-        <v>0.001</v>
+        <v>0.0012</v>
       </c>
       <c r="N41" s="10">
         <f>IF(D41="Govt",$B$1,$B$2)</f>
@@ -2952,23 +2952,23 @@
         <v/>
       </c>
       <c r="Q41" s="12" t="n">
-        <v>5.2074</v>
+        <v>10.2901</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>BNP Paribas</t>
+          <t>Invesco</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>BNP PARIBAS EASY ESG ENHANCED EUR CORP BOND DECEMBER 2029 UCITS ETF C</t>
+          <t>Invesco BulletShares 2028 EUR Corporate Bond UCITS ETF Acc</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>LU2823896811</t>
+          <t>IE00079EUF59</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
@@ -2982,14 +2982,14 @@
         </is>
       </c>
       <c r="F42" s="6" t="n">
-        <v>47483</v>
+        <v>47118</v>
       </c>
       <c r="G42" s="7">
         <f>IF(F42="","",MAX(0,YEARFRAC(TODAY(),F42)))</f>
         <v/>
       </c>
       <c r="H42" s="8" t="n">
-        <v>0.0235</v>
+        <v>0.0242</v>
       </c>
       <c r="I42" s="8" t="n">
         <v>0.0383</v>
@@ -3000,7 +3000,7 @@
       <c r="K42" s="9" t="n"/>
       <c r="L42" s="9" t="n"/>
       <c r="M42" s="8" t="n">
-        <v>0.0012</v>
+        <v>0.001</v>
       </c>
       <c r="N42" s="10">
         <f>IF(D42="Govt",$B$1,$B$2)</f>
@@ -3015,23 +3015,23 @@
         <v/>
       </c>
       <c r="Q42" s="12" t="n">
-        <v>10.655</v>
+        <v>5.5692</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>BNP Paribas</t>
+          <t>Invesco</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>BNP PARIBAS EASY ESG ENHANCED EUR CORP BOND DECEMBER 2029 UCITS ETF D</t>
+          <t>Invesco BulletShares 2028 EUR Corporate Bond UCITS ETF Dist</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>LU2823896738</t>
+          <t>IE000LKGEZQ6</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
@@ -3045,14 +3045,14 @@
         </is>
       </c>
       <c r="F43" s="6" t="n">
-        <v>47483</v>
+        <v>47118</v>
       </c>
       <c r="G43" s="7">
         <f>IF(F43="","",MAX(0,YEARFRAC(TODAY(),F43)))</f>
         <v/>
       </c>
       <c r="H43" s="8" t="n">
-        <v>0.0235</v>
+        <v>0.0242</v>
       </c>
       <c r="I43" s="8" t="n">
         <v>0.0383</v>
@@ -3063,7 +3063,7 @@
       <c r="K43" s="9" t="n"/>
       <c r="L43" s="9" t="n"/>
       <c r="M43" s="8" t="n">
-        <v>0.0012</v>
+        <v>0.001</v>
       </c>
       <c r="N43" s="10">
         <f>IF(D43="Govt",$B$1,$B$2)</f>
@@ -3078,7 +3078,7 @@
         <v/>
       </c>
       <c r="Q43" s="12" t="n">
-        <v>10.2938</v>
+        <v>5.2086</v>
       </c>
     </row>
     <row r="44">
@@ -3118,10 +3118,10 @@
         <v>0.0214</v>
       </c>
       <c r="I44" s="8" t="n">
-        <v>0.0371</v>
+        <v>0.0373</v>
       </c>
       <c r="J44" s="9" t="n">
-        <v>0</v>
+        <v>0.0002</v>
       </c>
       <c r="K44" s="9" t="n"/>
       <c r="L44" s="9" t="n"/>
@@ -3147,22 +3147,22 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>DWS</t>
+          <t>Amundi</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Xtrackers II Target Maturity Sept 2028 EUR Corporate Bond UCITS ETF 1D</t>
+          <t>Amundi Fixed Maturity 2027 Italy BTP Government Bond UCITS ETF Dist</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>LU2810185665</t>
+          <t>LU2780872128</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>Corp</t>
+          <t>Govt</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -3171,25 +3171,25 @@
         </is>
       </c>
       <c r="F45" s="6" t="n">
-        <v>47026</v>
+        <v>46752</v>
       </c>
       <c r="G45" s="7">
         <f>IF(F45="","",MAX(0,YEARFRAC(TODAY(),F45)))</f>
         <v/>
       </c>
       <c r="H45" s="8" t="n">
-        <v>0.0207</v>
+        <v>0.0265</v>
       </c>
       <c r="I45" s="8" t="n">
-        <v>0.0366</v>
+        <v>0.0313</v>
       </c>
       <c r="J45" s="9" t="n">
-        <v>0.0004</v>
+        <v>0.0008</v>
       </c>
       <c r="K45" s="9" t="n"/>
       <c r="L45" s="9" t="n"/>
       <c r="M45" s="8" t="n">
-        <v>0.0012</v>
+        <v>0.0009</v>
       </c>
       <c r="N45" s="10">
         <f>IF(D45="Govt",$B$1,$B$2)</f>
@@ -3204,28 +3204,28 @@
         <v/>
       </c>
       <c r="Q45" s="12" t="n">
-        <v>35.75</v>
+        <v>10.3323</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Amundi</t>
+          <t>DWS</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Amundi Fixed Maturity 2027 Italy BTP Government Bond UCITS ETF Dist</t>
+          <t>Xtrackers II Target Maturity Sept 2028 EUR Corporate Bond UCITS ETF 1D</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>LU2780872128</t>
+          <t>LU2810185665</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>Govt</t>
+          <t>Corp</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -3234,25 +3234,25 @@
         </is>
       </c>
       <c r="F46" s="6" t="n">
-        <v>46752</v>
+        <v>47026</v>
       </c>
       <c r="G46" s="7">
         <f>IF(F46="","",MAX(0,YEARFRAC(TODAY(),F46)))</f>
         <v/>
       </c>
       <c r="H46" s="8" t="n">
-        <v>0.0265</v>
+        <v>0.0207</v>
       </c>
       <c r="I46" s="8" t="n">
-        <v>0.0305</v>
+        <v>0.0368</v>
       </c>
       <c r="J46" s="9" t="n">
-        <v>-0.0002</v>
+        <v>0.0002</v>
       </c>
       <c r="K46" s="9" t="n"/>
       <c r="L46" s="9" t="n"/>
       <c r="M46" s="8" t="n">
-        <v>0.0009</v>
+        <v>0.0012</v>
       </c>
       <c r="N46" s="10">
         <f>IF(D46="Govt",$B$1,$B$2)</f>
@@ -3267,7 +3267,7 @@
         <v/>
       </c>
       <c r="Q46" s="12" t="n">
-        <v>10.3289</v>
+        <v>35.75</v>
       </c>
     </row>
     <row r="47">
@@ -3307,10 +3307,10 @@
         <v>0.015</v>
       </c>
       <c r="I47" s="8" t="n">
-        <v>0.0299</v>
+        <v>0.0296</v>
       </c>
       <c r="J47" s="9" t="n">
-        <v>-0.0001</v>
+        <v>-0.0003</v>
       </c>
       <c r="K47" s="9" t="n"/>
       <c r="L47" s="9" t="n"/>
@@ -3330,7 +3330,7 @@
         <v/>
       </c>
       <c r="Q47" s="12" t="n">
-        <v>10.1703</v>
+        <v>10.1716</v>
       </c>
     </row>
     <row r="48">
@@ -3341,12 +3341,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Amundi Fixed Maturity 2026 Euro Government Bond Broad UCITS ETF Acc</t>
+          <t>Amundi Fixed Maturity 2027 German Bund Government Bond UCITS ETF Dist</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>LU2872291278</t>
+          <t>LU2780871823</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
@@ -3356,24 +3356,24 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>Acc</t>
+          <t>Dist</t>
         </is>
       </c>
       <c r="F48" s="6" t="n">
-        <v>46387</v>
+        <v>46752</v>
       </c>
       <c r="G48" s="7">
         <f>IF(F48="","",MAX(0,YEARFRAC(TODAY(),F48)))</f>
         <v/>
       </c>
       <c r="H48" s="8" t="n">
-        <v>0.0023</v>
+        <v>0.0105</v>
       </c>
       <c r="I48" s="8" t="n">
-        <v>0.0293</v>
+        <v>0.0284</v>
       </c>
       <c r="J48" s="9" t="n">
-        <v>0.003</v>
+        <v>-0.0008</v>
       </c>
       <c r="K48" s="9" t="n"/>
       <c r="L48" s="9" t="n"/>
@@ -3393,33 +3393,33 @@
         <v/>
       </c>
       <c r="Q48" s="12" t="n">
-        <v>10.2535</v>
+        <v>10.3434</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Amundi</t>
+          <t>iShares</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Amundi Fixed Maturity 2027 German Bund Government Bond UCITS ETF Dist</t>
+          <t>iShares iBonds Dec 2027 Term € Corp UCITS ETF</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>LU2780871823</t>
+          <t>IE000ZOI8OK5</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>Govt</t>
+          <t>Corp</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>Dist</t>
+          <t>Acc</t>
         </is>
       </c>
       <c r="F49" s="6" t="n">
@@ -3430,18 +3430,18 @@
         <v/>
       </c>
       <c r="H49" s="8" t="n">
-        <v>0.0105</v>
+        <v>0.0195</v>
       </c>
       <c r="I49" s="8" t="n">
-        <v>0.0292</v>
+        <v>0.0333</v>
       </c>
       <c r="J49" s="9" t="n">
-        <v>-0.0001</v>
+        <v>0.0001</v>
       </c>
       <c r="K49" s="9" t="n"/>
       <c r="L49" s="9" t="n"/>
       <c r="M49" s="8" t="n">
-        <v>0.0009</v>
+        <v>0.0012</v>
       </c>
       <c r="N49" s="10">
         <f>IF(D49="Govt",$B$1,$B$2)</f>
@@ -3456,7 +3456,7 @@
         <v/>
       </c>
       <c r="Q49" s="12" t="n">
-        <v>10.3443</v>
+        <v>5.65</v>
       </c>
     </row>
     <row r="50">
@@ -3519,7 +3519,7 @@
         <v/>
       </c>
       <c r="Q50" s="12" t="n">
-        <v>5.7041</v>
+        <v>5.7046</v>
       </c>
     </row>
     <row r="51">
@@ -3582,23 +3582,23 @@
         <v/>
       </c>
       <c r="Q51" s="12" t="n">
-        <v>5.332</v>
+        <v>5.3325</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>iShares</t>
+          <t>DWS</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>iShares iBonds Dec 2027 Term € Corp UCITS ETF</t>
+          <t>Xtrackers II Target Maturity Sept 2027 EUR Corporate Bond UCITS ETF 1D</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>IE000ZOI8OK5</t>
+          <t>LU2673523218</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
@@ -3608,24 +3608,24 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>Acc</t>
+          <t>Dist</t>
         </is>
       </c>
       <c r="F52" s="6" t="n">
-        <v>46752</v>
+        <v>46660</v>
       </c>
       <c r="G52" s="7">
         <f>IF(F52="","",MAX(0,YEARFRAC(TODAY(),F52)))</f>
         <v/>
       </c>
       <c r="H52" s="8" t="n">
-        <v>0.0195</v>
+        <v>0.0187</v>
       </c>
       <c r="I52" s="8" t="n">
-        <v>0.0332</v>
+        <v>0.0325</v>
       </c>
       <c r="J52" s="9" t="n">
-        <v>0</v>
+        <v>0.0005</v>
       </c>
       <c r="K52" s="9" t="n"/>
       <c r="L52" s="9" t="n"/>
@@ -3645,7 +3645,7 @@
         <v/>
       </c>
       <c r="Q52" s="12" t="n">
-        <v>5.65</v>
+        <v>25.95</v>
       </c>
     </row>
     <row r="53">
@@ -3656,12 +3656,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Xtrackers II Target Maturity Sept 2027 EUR Corporate Bond UCITS ETF 1D</t>
+          <t>Xtrackers II Target Maturity Sept 2027 EUR Corporate Bond UCITS ETF 1C</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>LU2673523218</t>
+          <t>LU2673522830</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
@@ -3671,7 +3671,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t>Dist</t>
+          <t>Acc</t>
         </is>
       </c>
       <c r="F53" s="6" t="n">
@@ -3682,13 +3682,13 @@
         <v/>
       </c>
       <c r="H53" s="8" t="n">
-        <v>0.0186</v>
+        <v>0.0187</v>
       </c>
       <c r="I53" s="8" t="n">
-        <v>0.032</v>
+        <v>0.0325</v>
       </c>
       <c r="J53" s="9" t="n">
-        <v>0.0063</v>
+        <v>0.0005</v>
       </c>
       <c r="K53" s="9" t="n"/>
       <c r="L53" s="9" t="n"/>
@@ -3708,50 +3708,50 @@
         <v/>
       </c>
       <c r="Q53" s="12" t="n">
-        <v>25.94</v>
+        <v>9.300000000000001</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>DWS</t>
+          <t>iShares</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Xtrackers II Target Maturity Sept 2027 EUR Corporate Bond UCITS ETF 1C</t>
+          <t>iShares iBonds Dec 2026 Term € Italy Govt Bond UCITS ETF</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>LU2673522830</t>
+          <t>IE000LZ7BZW8</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>Corp</t>
+          <t>Govt</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t>Acc</t>
+          <t>Dist</t>
         </is>
       </c>
       <c r="F54" s="6" t="n">
-        <v>46660</v>
+        <v>46387</v>
       </c>
       <c r="G54" s="7">
         <f>IF(F54="","",MAX(0,YEARFRAC(TODAY(),F54)))</f>
         <v/>
       </c>
       <c r="H54" s="8" t="n">
-        <v>0.0186</v>
+        <v>0.008800000000000001</v>
       </c>
       <c r="I54" s="8" t="n">
-        <v>0.032</v>
+        <v>0.0272</v>
       </c>
       <c r="J54" s="9" t="n">
-        <v>0.0063</v>
+        <v>0.0002</v>
       </c>
       <c r="K54" s="9" t="n"/>
       <c r="L54" s="9" t="n"/>
@@ -3771,23 +3771,23 @@
         <v/>
       </c>
       <c r="Q54" s="12" t="n">
-        <v>9.300000000000001</v>
+        <v>5.06</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>iShares</t>
+          <t>Amundi</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>iShares iBonds Dec 2026 Term € Italy Govt Bond UCITS ETF</t>
+          <t>Amundi Fixed Maturity 2026 Euro Government Bond Broad UCITS ETF Acc</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>IE000LZ7BZW8</t>
+          <t>LU2872291278</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
@@ -3797,7 +3797,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t>Dist</t>
+          <t>Acc</t>
         </is>
       </c>
       <c r="F55" s="6" t="n">
@@ -3808,18 +3808,18 @@
         <v/>
       </c>
       <c r="H55" s="8" t="n">
-        <v>0.008800000000000001</v>
+        <v>0.0023</v>
       </c>
       <c r="I55" s="8" t="n">
-        <v>0.027</v>
+        <v>0.0261</v>
       </c>
       <c r="J55" s="9" t="n">
-        <v>0</v>
+        <v>-0.0032</v>
       </c>
       <c r="K55" s="9" t="n"/>
       <c r="L55" s="9" t="n"/>
       <c r="M55" s="8" t="n">
-        <v>0.0012</v>
+        <v>0.0009</v>
       </c>
       <c r="N55" s="10">
         <f>IF(D55="Govt",$B$1,$B$2)</f>
@@ -3834,7 +3834,7 @@
         <v/>
       </c>
       <c r="Q55" s="12" t="n">
-        <v>5.06</v>
+        <v>10.2545</v>
       </c>
     </row>
     <row r="56">
@@ -3897,7 +3897,7 @@
         <v/>
       </c>
       <c r="Q56" s="12" t="n">
-        <v>5.7887</v>
+        <v>5.7896</v>
       </c>
     </row>
     <row r="57">
@@ -3960,7 +3960,7 @@
         <v/>
       </c>
       <c r="Q57" s="12" t="n">
-        <v>5.4127</v>
+        <v>5.4135</v>
       </c>
     </row>
     <row r="58">
@@ -3997,13 +3997,13 @@
         <v/>
       </c>
       <c r="H58" s="8" t="n">
-        <v>0.0061</v>
+        <v>0.0063</v>
       </c>
       <c r="I58" s="8" t="n">
-        <v>0.0278</v>
+        <v>0.0283</v>
       </c>
       <c r="J58" s="9" t="n">
-        <v>0</v>
+        <v>0.0005</v>
       </c>
       <c r="K58" s="9" t="n"/>
       <c r="L58" s="9" t="n"/>

</xml_diff>

<commit_message>
Aggiorna yield_etf 13/10/2026; controllo completezza su ISIN distinti (due giri nello stesso giorno non lo falsano), rimosso duplicato 12/10
</commit_message>
<xml_diff>
--- a/data/rendimenti_etf.xlsx
+++ b/data/rendimenti_etf.xlsx
@@ -533,7 +533,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Aggiornato il 12/10/2026 14:48 da yield_etf.csv</t>
+          <t>Aggiornato il 13/10/2026 09:32 da yield_etf.csv</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
         <v>0.0501</v>
       </c>
       <c r="J5" s="9" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0</v>
       </c>
       <c r="K5" s="9" t="n"/>
       <c r="L5" s="9" t="n"/>
@@ -727,7 +727,7 @@
         <v>0.0462</v>
       </c>
       <c r="J6" s="9" t="n">
-        <v>-0.0001</v>
+        <v>0</v>
       </c>
       <c r="K6" s="9" t="n"/>
       <c r="L6" s="9" t="n"/>
@@ -790,7 +790,7 @@
         <v>0.0459</v>
       </c>
       <c r="J7" s="9" t="n">
-        <v>-0.0001</v>
+        <v>0</v>
       </c>
       <c r="K7" s="9" t="n"/>
       <c r="L7" s="9" t="n"/>
@@ -810,7 +810,7 @@
         <v/>
       </c>
       <c r="Q7" s="12" t="n">
-        <v>4.81</v>
+        <v>4.82</v>
       </c>
     </row>
     <row r="8">
@@ -853,7 +853,7 @@
         <v>0.0458</v>
       </c>
       <c r="J8" s="9" t="n">
-        <v>-0.0001</v>
+        <v>0</v>
       </c>
       <c r="K8" s="9" t="n"/>
       <c r="L8" s="9" t="n"/>
@@ -916,7 +916,7 @@
         <v>0.0457</v>
       </c>
       <c r="J9" s="9" t="n">
-        <v>-0.0001</v>
+        <v>0</v>
       </c>
       <c r="K9" s="9" t="n"/>
       <c r="L9" s="9" t="n"/>
@@ -936,7 +936,7 @@
         <v/>
       </c>
       <c r="Q9" s="12" t="n">
-        <v>4.8</v>
+        <v>4.81</v>
       </c>
     </row>
     <row r="10">
@@ -979,7 +979,7 @@
         <v>0.0455</v>
       </c>
       <c r="J10" s="9" t="n">
-        <v>-0.0001</v>
+        <v>0</v>
       </c>
       <c r="K10" s="9" t="n"/>
       <c r="L10" s="9" t="n"/>
@@ -999,7 +999,7 @@
         <v/>
       </c>
       <c r="Q10" s="12" t="n">
-        <v>4.72</v>
+        <v>4.73</v>
       </c>
     </row>
     <row r="11">
@@ -1231,7 +1231,7 @@
         <v>0.044</v>
       </c>
       <c r="J14" s="9" t="n">
-        <v>0.0005</v>
+        <v>0</v>
       </c>
       <c r="K14" s="9" t="n"/>
       <c r="L14" s="9" t="n"/>
@@ -1294,7 +1294,7 @@
         <v>0.044</v>
       </c>
       <c r="J15" s="9" t="n">
-        <v>0.0005</v>
+        <v>0</v>
       </c>
       <c r="K15" s="9" t="n"/>
       <c r="L15" s="9" t="n"/>
@@ -1357,7 +1357,7 @@
         <v>0.0444</v>
       </c>
       <c r="J16" s="9" t="n">
-        <v>0.0005</v>
+        <v>0</v>
       </c>
       <c r="K16" s="9" t="n"/>
       <c r="L16" s="9" t="n"/>
@@ -1420,7 +1420,7 @@
         <v>0.0435</v>
       </c>
       <c r="J17" s="9" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
       <c r="K17" s="9" t="n"/>
       <c r="L17" s="9" t="n"/>
@@ -1483,7 +1483,7 @@
         <v>0.0429</v>
       </c>
       <c r="J18" s="9" t="n">
-        <v>0.0002</v>
+        <v>0</v>
       </c>
       <c r="K18" s="9" t="n"/>
       <c r="L18" s="9" t="n"/>
@@ -1509,41 +1509,41 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>iShares</t>
+          <t>Amundi</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>iShares iBonds Dec 2031 Term € Corp UCITS ETF</t>
+          <t>Amundi Fixed Maturity 2030 Euro Government Bond Broad UCITS ETF Acc</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>IE000I2WYEU9</t>
+          <t>LU3120976132</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Corp</t>
+          <t>Govt</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Dist</t>
+          <t>Acc</t>
         </is>
       </c>
       <c r="F19" s="6" t="n">
-        <v>48213</v>
+        <v>47848</v>
       </c>
       <c r="G19" s="7">
         <f>IF(F19="","",MAX(0,YEARFRAC(TODAY(),F19)))</f>
         <v/>
       </c>
       <c r="H19" s="8" t="n">
-        <v>0.0285</v>
+        <v>0.0169</v>
       </c>
       <c r="I19" s="8" t="n">
-        <v>0.04219999999999999</v>
+        <v>0.0357</v>
       </c>
       <c r="J19" s="9" t="n">
         <v>0.0002</v>
@@ -1551,7 +1551,7 @@
       <c r="K19" s="9" t="n"/>
       <c r="L19" s="9" t="n"/>
       <c r="M19" s="8" t="n">
-        <v>0.0012</v>
+        <v>0.0009</v>
       </c>
       <c r="N19" s="10">
         <f>IF(D19="Govt",$B$1,$B$2)</f>
@@ -1566,55 +1566,55 @@
         <v/>
       </c>
       <c r="Q19" s="12" t="n">
-        <v>4.87</v>
+        <v>9.8248</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Amundi</t>
+          <t>iShares</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Amundi Fixed Maturity 2030 Euro Government Bond Broad UCITS ETF Acc</t>
+          <t>iShares iBonds Dec 2031 Term € Corp UCITS ETF</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>LU3120976132</t>
+          <t>IE000I2WYEU9</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Govt</t>
+          <t>Corp</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Acc</t>
+          <t>Dist</t>
         </is>
       </c>
       <c r="F20" s="6" t="n">
-        <v>47848</v>
+        <v>48213</v>
       </c>
       <c r="G20" s="7">
         <f>IF(F20="","",MAX(0,YEARFRAC(TODAY(),F20)))</f>
         <v/>
       </c>
       <c r="H20" s="8" t="n">
-        <v>0.0169</v>
+        <v>0.0285</v>
       </c>
       <c r="I20" s="8" t="n">
-        <v>0.0355</v>
+        <v>0.04219999999999999</v>
       </c>
       <c r="J20" s="9" t="n">
-        <v>-0.0007</v>
+        <v>0</v>
       </c>
       <c r="K20" s="9" t="n"/>
       <c r="L20" s="9" t="n"/>
       <c r="M20" s="8" t="n">
-        <v>0.0009</v>
+        <v>0.0012</v>
       </c>
       <c r="N20" s="10">
         <f>IF(D20="Govt",$B$1,$B$2)</f>
@@ -1629,7 +1629,7 @@
         <v/>
       </c>
       <c r="Q20" s="12" t="n">
-        <v>9.830500000000001</v>
+        <v>4.87</v>
       </c>
     </row>
     <row r="21">
@@ -1672,7 +1672,7 @@
         <v>0.0421</v>
       </c>
       <c r="J21" s="9" t="n">
-        <v>0.0002</v>
+        <v>0</v>
       </c>
       <c r="K21" s="9" t="n"/>
       <c r="L21" s="9" t="n"/>
@@ -1735,7 +1735,7 @@
         <v>0.0421</v>
       </c>
       <c r="J22" s="9" t="n">
-        <v>0.0002</v>
+        <v>0</v>
       </c>
       <c r="K22" s="9" t="n"/>
       <c r="L22" s="9" t="n"/>
@@ -1798,7 +1798,7 @@
         <v>0.04190000000000001</v>
       </c>
       <c r="J23" s="9" t="n">
-        <v>0.0002</v>
+        <v>0</v>
       </c>
       <c r="K23" s="9" t="n"/>
       <c r="L23" s="9" t="n"/>
@@ -1861,7 +1861,7 @@
         <v>0.04190000000000001</v>
       </c>
       <c r="J24" s="9" t="n">
-        <v>0.0002</v>
+        <v>0</v>
       </c>
       <c r="K24" s="9" t="n"/>
       <c r="L24" s="9" t="n"/>
@@ -1921,10 +1921,10 @@
         <v>0.0208</v>
       </c>
       <c r="I25" s="8" t="n">
-        <v>0.0346</v>
+        <v>0.0348</v>
       </c>
       <c r="J25" s="9" t="n">
-        <v>-0.0007</v>
+        <v>0.0002</v>
       </c>
       <c r="K25" s="9" t="n"/>
       <c r="L25" s="9" t="n"/>
@@ -1944,7 +1944,7 @@
         <v/>
       </c>
       <c r="Q25" s="12" t="n">
-        <v>9.985900000000001</v>
+        <v>9.9818</v>
       </c>
     </row>
     <row r="26">
@@ -1987,7 +1987,7 @@
         <v>0.0349</v>
       </c>
       <c r="J26" s="9" t="n">
-        <v>0.0002</v>
+        <v>0</v>
       </c>
       <c r="K26" s="9" t="n"/>
       <c r="L26" s="9" t="n"/>
@@ -2070,7 +2070,7 @@
         <v/>
       </c>
       <c r="Q27" s="12" t="n">
-        <v>5.3493</v>
+        <v>5.35</v>
       </c>
     </row>
     <row r="28">
@@ -2133,7 +2133,7 @@
         <v/>
       </c>
       <c r="Q28" s="12" t="n">
-        <v>4.9828</v>
+        <v>4.9834</v>
       </c>
     </row>
     <row r="29">
@@ -2176,7 +2176,7 @@
         <v>0.0406</v>
       </c>
       <c r="J29" s="9" t="n">
-        <v>0.0003</v>
+        <v>0</v>
       </c>
       <c r="K29" s="9" t="n"/>
       <c r="L29" s="9" t="n"/>
@@ -2239,7 +2239,7 @@
         <v>0.0405</v>
       </c>
       <c r="J30" s="9" t="n">
-        <v>0.0003</v>
+        <v>0</v>
       </c>
       <c r="K30" s="9" t="n"/>
       <c r="L30" s="9" t="n"/>
@@ -2302,7 +2302,7 @@
         <v>0.034</v>
       </c>
       <c r="J31" s="9" t="n">
-        <v>0.0003</v>
+        <v>0</v>
       </c>
       <c r="K31" s="9" t="n"/>
       <c r="L31" s="9" t="n"/>
@@ -2359,13 +2359,13 @@
         <v/>
       </c>
       <c r="H32" s="8" t="n">
-        <v>0.023</v>
+        <v>0.0229</v>
       </c>
       <c r="I32" s="8" t="n">
-        <v>0.0328</v>
+        <v>0.0329</v>
       </c>
       <c r="J32" s="9" t="n">
-        <v>-0.0004</v>
+        <v>0.0001</v>
       </c>
       <c r="K32" s="9" t="n"/>
       <c r="L32" s="9" t="n"/>
@@ -2385,7 +2385,7 @@
         <v/>
       </c>
       <c r="Q32" s="12" t="n">
-        <v>10.285</v>
+        <v>10.2821</v>
       </c>
     </row>
     <row r="33">
@@ -2428,7 +2428,7 @@
         <v>0.0389</v>
       </c>
       <c r="J33" s="9" t="n">
-        <v>0.0004</v>
+        <v>0</v>
       </c>
       <c r="K33" s="9" t="n"/>
       <c r="L33" s="9" t="n"/>
@@ -2448,7 +2448,7 @@
         <v/>
       </c>
       <c r="Q33" s="12" t="n">
-        <v>5.04</v>
+        <v>5.03</v>
       </c>
     </row>
     <row r="34">
@@ -2511,7 +2511,7 @@
         <v/>
       </c>
       <c r="Q34" s="12" t="n">
-        <v>5.4253</v>
+        <v>5.4251</v>
       </c>
     </row>
     <row r="35">
@@ -2574,28 +2574,28 @@
         <v/>
       </c>
       <c r="Q35" s="12" t="n">
-        <v>5.0554</v>
+        <v>5.0552</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>DWS</t>
+          <t>Amundi</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Xtrackers II Target Maturity Sept 2029 EUR Corporate Bond UCITS ETF 1D</t>
+          <t>Amundi Fixed Maturity 2028 Euro Government Bond Broad UCITS ETF Dist</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>LU2673523309</t>
+          <t>LU2780871401</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Corp</t>
+          <t>Govt</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -2604,25 +2604,25 @@
         </is>
       </c>
       <c r="F36" s="6" t="n">
-        <v>47391</v>
+        <v>47118</v>
       </c>
       <c r="G36" s="7">
         <f>IF(F36="","",MAX(0,YEARFRAC(TODAY(),F36)))</f>
         <v/>
       </c>
       <c r="H36" s="8" t="n">
-        <v>0.0245</v>
+        <v>0.0184</v>
       </c>
       <c r="I36" s="8" t="n">
-        <v>0.0386</v>
+        <v>0.0326</v>
       </c>
       <c r="J36" s="9" t="n">
-        <v>0.0004</v>
+        <v>0.0001</v>
       </c>
       <c r="K36" s="9" t="n"/>
       <c r="L36" s="9" t="n"/>
       <c r="M36" s="8" t="n">
-        <v>0.0012</v>
+        <v>0.0009</v>
       </c>
       <c r="N36" s="10">
         <f>IF(D36="Govt",$B$1,$B$2)</f>
@@ -2637,28 +2637,28 @@
         <v/>
       </c>
       <c r="Q36" s="12" t="n">
-        <v>25.78</v>
+        <v>10.2724</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>DWS</t>
+          <t>Amundi</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Xtrackers II Target Maturity Sept 2029 EUR Corporate Bond UCITS ETF 1C</t>
+          <t>Amundi Fixed Maturity 2028 Euro Government Bond Broad UCITS ETF Acc</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>LU2673522913</t>
+          <t>LU2780871310</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Corp</t>
+          <t>Govt</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -2667,25 +2667,25 @@
         </is>
       </c>
       <c r="F37" s="6" t="n">
-        <v>47391</v>
+        <v>47118</v>
       </c>
       <c r="G37" s="7">
         <f>IF(F37="","",MAX(0,YEARFRAC(TODAY(),F37)))</f>
         <v/>
       </c>
       <c r="H37" s="8" t="n">
-        <v>0.0245</v>
+        <v>0.0184</v>
       </c>
       <c r="I37" s="8" t="n">
-        <v>0.0386</v>
+        <v>0.0326</v>
       </c>
       <c r="J37" s="9" t="n">
-        <v>0.0004</v>
+        <v>0.0001</v>
       </c>
       <c r="K37" s="9" t="n"/>
       <c r="L37" s="9" t="n"/>
       <c r="M37" s="8" t="n">
-        <v>0.0012</v>
+        <v>0.0009</v>
       </c>
       <c r="N37" s="10">
         <f>IF(D37="Govt",$B$1,$B$2)</f>
@@ -2700,28 +2700,28 @@
         <v/>
       </c>
       <c r="Q37" s="12" t="n">
-        <v>9.17</v>
+        <v>10.0719</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Amundi</t>
+          <t>DWS</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Amundi Fixed Maturity 2028 Euro Government Bond Broad UCITS ETF Dist</t>
+          <t>Xtrackers II Target Maturity Sept 2029 EUR Corporate Bond UCITS ETF 1D</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>LU2780871401</t>
+          <t>LU2673523309</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Govt</t>
+          <t>Corp</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -2730,25 +2730,25 @@
         </is>
       </c>
       <c r="F38" s="6" t="n">
-        <v>47118</v>
+        <v>47391</v>
       </c>
       <c r="G38" s="7">
         <f>IF(F38="","",MAX(0,YEARFRAC(TODAY(),F38)))</f>
         <v/>
       </c>
       <c r="H38" s="8" t="n">
-        <v>0.0184</v>
+        <v>0.0245</v>
       </c>
       <c r="I38" s="8" t="n">
-        <v>0.0325</v>
+        <v>0.0386</v>
       </c>
       <c r="J38" s="9" t="n">
-        <v>-0.0003</v>
+        <v>0</v>
       </c>
       <c r="K38" s="9" t="n"/>
       <c r="L38" s="9" t="n"/>
       <c r="M38" s="8" t="n">
-        <v>0.0009</v>
+        <v>0.0012</v>
       </c>
       <c r="N38" s="10">
         <f>IF(D38="Govt",$B$1,$B$2)</f>
@@ -2763,28 +2763,28 @@
         <v/>
       </c>
       <c r="Q38" s="12" t="n">
-        <v>10.2754</v>
+        <v>25.78</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Amundi</t>
+          <t>DWS</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Amundi Fixed Maturity 2028 Euro Government Bond Broad UCITS ETF Acc</t>
+          <t>Xtrackers II Target Maturity Sept 2029 EUR Corporate Bond UCITS ETF 1C</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>LU2780871310</t>
+          <t>LU2673522913</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Govt</t>
+          <t>Corp</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -2793,25 +2793,25 @@
         </is>
       </c>
       <c r="F39" s="6" t="n">
-        <v>47118</v>
+        <v>47391</v>
       </c>
       <c r="G39" s="7">
         <f>IF(F39="","",MAX(0,YEARFRAC(TODAY(),F39)))</f>
         <v/>
       </c>
       <c r="H39" s="8" t="n">
-        <v>0.0184</v>
+        <v>0.0245</v>
       </c>
       <c r="I39" s="8" t="n">
-        <v>0.0325</v>
+        <v>0.0386</v>
       </c>
       <c r="J39" s="9" t="n">
-        <v>-0.0003</v>
+        <v>0</v>
       </c>
       <c r="K39" s="9" t="n"/>
       <c r="L39" s="9" t="n"/>
       <c r="M39" s="8" t="n">
-        <v>0.0009</v>
+        <v>0.0012</v>
       </c>
       <c r="N39" s="10">
         <f>IF(D39="Govt",$B$1,$B$2)</f>
@@ -2826,7 +2826,7 @@
         <v/>
       </c>
       <c r="Q39" s="12" t="n">
-        <v>10.0748</v>
+        <v>9.17</v>
       </c>
     </row>
     <row r="40">
@@ -2869,7 +2869,7 @@
         <v>0.0382</v>
       </c>
       <c r="J40" s="9" t="n">
-        <v>0.0003</v>
+        <v>0</v>
       </c>
       <c r="K40" s="9" t="n"/>
       <c r="L40" s="9" t="n"/>
@@ -2932,7 +2932,7 @@
         <v>0.0382</v>
       </c>
       <c r="J41" s="9" t="n">
-        <v>0.0003</v>
+        <v>0</v>
       </c>
       <c r="K41" s="9" t="n"/>
       <c r="L41" s="9" t="n"/>
@@ -3015,7 +3015,7 @@
         <v/>
       </c>
       <c r="Q42" s="12" t="n">
-        <v>5.5695</v>
+        <v>5.5691</v>
       </c>
     </row>
     <row r="43">
@@ -3078,7 +3078,7 @@
         <v/>
       </c>
       <c r="Q43" s="12" t="n">
-        <v>5.2089</v>
+        <v>5.2084</v>
       </c>
     </row>
     <row r="44">
@@ -3121,7 +3121,7 @@
         <v>0.0373</v>
       </c>
       <c r="J44" s="9" t="n">
-        <v>0.0003</v>
+        <v>0</v>
       </c>
       <c r="K44" s="9" t="n"/>
       <c r="L44" s="9" t="n"/>
@@ -3184,7 +3184,7 @@
         <v>0.0369</v>
       </c>
       <c r="J45" s="9" t="n">
-        <v>0.0002</v>
+        <v>0</v>
       </c>
       <c r="K45" s="9" t="n"/>
       <c r="L45" s="9" t="n"/>
@@ -3244,10 +3244,10 @@
         <v>0.0265</v>
       </c>
       <c r="I46" s="8" t="n">
-        <v>0.0305</v>
+        <v>0.0306</v>
       </c>
       <c r="J46" s="9" t="n">
-        <v>-0.0002</v>
+        <v>0.0001</v>
       </c>
       <c r="K46" s="9" t="n"/>
       <c r="L46" s="9" t="n"/>
@@ -3267,7 +3267,7 @@
         <v/>
       </c>
       <c r="Q46" s="12" t="n">
-        <v>10.3332</v>
+        <v>10.3321</v>
       </c>
     </row>
     <row r="47">
@@ -3307,10 +3307,10 @@
         <v>0.015</v>
       </c>
       <c r="I47" s="8" t="n">
-        <v>0.0294</v>
+        <v>0.0295</v>
       </c>
       <c r="J47" s="9" t="n">
-        <v>-0.0001</v>
+        <v>0.0001</v>
       </c>
       <c r="K47" s="9" t="n"/>
       <c r="L47" s="9" t="n"/>
@@ -3330,7 +3330,7 @@
         <v/>
       </c>
       <c r="Q47" s="12" t="n">
-        <v>10.1744</v>
+        <v>10.1732</v>
       </c>
     </row>
     <row r="48">
@@ -3370,7 +3370,7 @@
         <v>0.0105</v>
       </c>
       <c r="I48" s="8" t="n">
-        <v>0.0284</v>
+        <v>0.0285</v>
       </c>
       <c r="J48" s="9" t="n">
         <v>0.0001</v>
@@ -3393,7 +3393,7 @@
         <v/>
       </c>
       <c r="Q48" s="12" t="n">
-        <v>10.3477</v>
+        <v>10.3462</v>
       </c>
     </row>
     <row r="49">
@@ -3456,7 +3456,7 @@
         <v/>
       </c>
       <c r="Q49" s="12" t="n">
-        <v>5.7061</v>
+        <v>5.7067</v>
       </c>
     </row>
     <row r="50">
@@ -3519,7 +3519,7 @@
         <v/>
       </c>
       <c r="Q50" s="12" t="n">
-        <v>5.3339</v>
+        <v>5.3344</v>
       </c>
     </row>
     <row r="51">
@@ -3588,49 +3588,49 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>DWS</t>
+          <t>Amundi</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Xtrackers II Target Maturity Sept 2027 EUR Corporate Bond UCITS ETF 1D</t>
+          <t>Amundi Fixed Maturity 2026 Euro Government Bond Broad UCITS ETF Acc</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>LU2673523218</t>
+          <t>LU2872291278</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>Corp</t>
+          <t>Govt</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>Dist</t>
+          <t>Acc</t>
         </is>
       </c>
       <c r="F52" s="6" t="n">
-        <v>46660</v>
+        <v>46387</v>
       </c>
       <c r="G52" s="7">
         <f>IF(F52="","",MAX(0,YEARFRAC(TODAY(),F52)))</f>
         <v/>
       </c>
       <c r="H52" s="8" t="n">
-        <v>0.0186</v>
+        <v>0.0023</v>
       </c>
       <c r="I52" s="8" t="n">
-        <v>0.032</v>
+        <v>0.0272</v>
       </c>
       <c r="J52" s="9" t="n">
-        <v>-0.0005</v>
+        <v>0.0008</v>
       </c>
       <c r="K52" s="9" t="n"/>
       <c r="L52" s="9" t="n"/>
       <c r="M52" s="8" t="n">
-        <v>0.0012</v>
+        <v>0.0009</v>
       </c>
       <c r="N52" s="10">
         <f>IF(D52="Govt",$B$1,$B$2)</f>
@@ -3645,7 +3645,7 @@
         <v/>
       </c>
       <c r="Q52" s="12" t="n">
-        <v>25.96</v>
+        <v>10.2587</v>
       </c>
     </row>
     <row r="53">
@@ -3656,12 +3656,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Xtrackers II Target Maturity Sept 2027 EUR Corporate Bond UCITS ETF 1C</t>
+          <t>Xtrackers II Target Maturity Sept 2027 EUR Corporate Bond UCITS ETF 1D</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>LU2673522830</t>
+          <t>LU2673523218</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
@@ -3671,7 +3671,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t>Acc</t>
+          <t>Dist</t>
         </is>
       </c>
       <c r="F53" s="6" t="n">
@@ -3688,7 +3688,7 @@
         <v>0.032</v>
       </c>
       <c r="J53" s="9" t="n">
-        <v>-0.0005</v>
+        <v>0</v>
       </c>
       <c r="K53" s="9" t="n"/>
       <c r="L53" s="9" t="n"/>
@@ -3708,50 +3708,50 @@
         <v/>
       </c>
       <c r="Q53" s="12" t="n">
-        <v>9.31</v>
+        <v>25.96</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>iShares</t>
+          <t>DWS</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>iShares iBonds Dec 2026 Term € Italy Govt Bond UCITS ETF</t>
+          <t>Xtrackers II Target Maturity Sept 2027 EUR Corporate Bond UCITS ETF 1C</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>IE000LZ7BZW8</t>
+          <t>LU2673522830</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>Govt</t>
+          <t>Corp</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t>Dist</t>
+          <t>Acc</t>
         </is>
       </c>
       <c r="F54" s="6" t="n">
-        <v>46387</v>
+        <v>46660</v>
       </c>
       <c r="G54" s="7">
         <f>IF(F54="","",MAX(0,YEARFRAC(TODAY(),F54)))</f>
         <v/>
       </c>
       <c r="H54" s="8" t="n">
-        <v>0.008800000000000001</v>
+        <v>0.0186</v>
       </c>
       <c r="I54" s="8" t="n">
-        <v>0.0269</v>
+        <v>0.032</v>
       </c>
       <c r="J54" s="9" t="n">
-        <v>-0.0001</v>
+        <v>0</v>
       </c>
       <c r="K54" s="9" t="n"/>
       <c r="L54" s="9" t="n"/>
@@ -3771,23 +3771,23 @@
         <v/>
       </c>
       <c r="Q54" s="12" t="n">
-        <v>5.06</v>
+        <v>9.31</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Amundi</t>
+          <t>iShares</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Amundi Fixed Maturity 2026 Euro Government Bond Broad UCITS ETF Acc</t>
+          <t>iShares iBonds Dec 2026 Term € Italy Govt Bond UCITS ETF</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>LU2872291278</t>
+          <t>IE000LZ7BZW8</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
@@ -3797,7 +3797,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t>Acc</t>
+          <t>Dist</t>
         </is>
       </c>
       <c r="F55" s="6" t="n">
@@ -3808,18 +3808,18 @@
         <v/>
       </c>
       <c r="H55" s="8" t="n">
-        <v>0.0023</v>
+        <v>0.008800000000000001</v>
       </c>
       <c r="I55" s="8" t="n">
-        <v>0.0264</v>
+        <v>0.0269</v>
       </c>
       <c r="J55" s="9" t="n">
-        <v>-0.0005</v>
+        <v>0</v>
       </c>
       <c r="K55" s="9" t="n"/>
       <c r="L55" s="9" t="n"/>
       <c r="M55" s="8" t="n">
-        <v>0.0009</v>
+        <v>0.0012</v>
       </c>
       <c r="N55" s="10">
         <f>IF(D55="Govt",$B$1,$B$2)</f>
@@ -3834,7 +3834,7 @@
         <v/>
       </c>
       <c r="Q55" s="12" t="n">
-        <v>10.258</v>
+        <v>5.06</v>
       </c>
     </row>
     <row r="56">
@@ -3897,7 +3897,7 @@
         <v/>
       </c>
       <c r="Q56" s="12" t="n">
-        <v>5.7916</v>
+        <v>5.7924</v>
       </c>
     </row>
     <row r="57">
@@ -3960,7 +3960,7 @@
         <v/>
       </c>
       <c r="Q57" s="12" t="n">
-        <v>5.4154</v>
+        <v>5.4161</v>
       </c>
     </row>
     <row r="58">
@@ -4003,7 +4003,7 @@
         <v>0.0273</v>
       </c>
       <c r="J58" s="9" t="n">
-        <v>-0.0008</v>
+        <v>0</v>
       </c>
       <c r="K58" s="9" t="n"/>
       <c r="L58" s="9" t="n"/>

</xml_diff>